<commit_message>
feat: ultimos cambios entrega cascada
</commit_message>
<xml_diff>
--- a/Entregables/Matriz-Comunicaciones-14-09.xlsx
+++ b/Entregables/Matriz-Comunicaciones-14-09.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://frbautneduar-my.sharepoint.com/personal/jomansilla_frba_utn_edu_ar/Documents/04-Cuarto-Año-2026/Administracion-De-Sistemas-De-Información/TPA/Entregables/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="128" documentId="11_F25DC773A252ABDACC1048BDA95E51B25BDE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2AD8BE5B-BD23-480A-90C4-A0C1B4D6A564}"/>
+  <xr:revisionPtr revIDLastSave="133" documentId="11_F25DC773A252ABDACC1048BDA95E51B25BDE58E7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{80209C54-4CD9-4739-AA61-E606EC0EFA59}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="480" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="84">
   <si>
     <t>Equipo completo + Sponsor + Comité Directivo</t>
   </si>
@@ -67,9 +67,6 @@
   </si>
   <si>
     <t>Diaria (15 min)</t>
-  </si>
-  <si>
-    <t>Standup / Seguimiento diario de equipo</t>
   </si>
   <si>
     <t>Una vez (inicio del proyecto)</t>
@@ -105,10 +102,6 @@
 cada reunión</t>
   </si>
   <si>
-    <t>Al cierre de
-cada sprint</t>
-  </si>
-  <si>
     <t>Líder de Proyecto
 + Product Owner</t>
   </si>
@@ -140,20 +133,12 @@
 Product Owner</t>
   </si>
   <si>
-    <t>Quincenal
-(cierre de sprint)</t>
-  </si>
-  <si>
     <t>Presentación
 Oral + Escrito</t>
   </si>
   <si>
     <t>Sponsor + PO +
 Equipo + Stakeholders clave</t>
-  </si>
-  <si>
-    <t>Reporte de Estado de Sprint
-(avance del sprint, demostraciones de funcionalidades)</t>
   </si>
   <si>
     <t>Responsable de
@@ -323,9 +308,6 @@
     </r>
   </si>
   <si>
-    <t>Retrospectiva bisemanal</t>
-  </si>
-  <si>
     <t>Reseña quincenal</t>
   </si>
   <si>
@@ -357,6 +339,18 @@
   </si>
   <si>
     <t>LP, ARQ, BE, FE, QA, DBA, SEC</t>
+  </si>
+  <si>
+    <t>Informe de avance del proyecto (demostraciones de funcionalidades)</t>
+  </si>
+  <si>
+    <t>Bisemanal</t>
+  </si>
+  <si>
+    <t>Reunión quincenal de revisión y mejora</t>
+  </si>
+  <si>
+    <t>Reunión diaria de seguimiento del equipo</t>
   </si>
 </sst>
 </file>
@@ -539,29 +533,29 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -860,320 +854,320 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
+      <c r="A1" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
+      <c r="A2" s="20" t="s">
+        <v>75</v>
+      </c>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="B3" s="21"/>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21"/>
+      <c r="A3" s="26" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
     </row>
     <row r="4" spans="1:6" ht="24" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>1</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="F6" s="12" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
-        <v>37</v>
+        <v>80</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>34</v>
+        <v>81</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F7" s="7" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="E8" s="13" t="s">
         <v>1</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="F9" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>25</v>
+        <v>81</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E11" s="11" t="s">
         <v>1</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="14" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="B12" s="15" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E13" s="11" t="s">
         <v>1</v>
       </c>
       <c r="F13" s="7" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="15" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E14" s="15" t="s">
         <v>1</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E15" s="7" t="s">
         <v>1</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
+      <c r="A17" s="23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="19"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="19"/>
     </row>
     <row r="18" spans="1:6" ht="24" x14ac:dyDescent="0.25">
-      <c r="A18" s="24" t="s">
-        <v>20</v>
+      <c r="A18" s="22" t="s">
+        <v>19</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D18" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
+      <c r="D18" s="22" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" s="21"/>
+      <c r="F18" s="21"/>
     </row>
     <row r="19" spans="1:6" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D19" s="22" t="s">
-        <v>81</v>
-      </c>
-      <c r="E19" s="21"/>
-      <c r="F19" s="21"/>
+      <c r="D19" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="E19" s="19"/>
+      <c r="F19" s="19"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>14</v>
+        <v>83</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>13</v>
@@ -1181,43 +1175,43 @@
       <c r="C20" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D20" s="20" t="s">
-        <v>83</v>
-      </c>
-      <c r="E20" s="21"/>
-      <c r="F20" s="21"/>
+      <c r="D20" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="E20" s="19"/>
+      <c r="F20" s="19"/>
     </row>
     <row r="21" spans="1:6" ht="21.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="B21" s="7" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D21" s="22" t="s">
+      <c r="D21" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
+      <c r="E21" s="19"/>
+      <c r="F21" s="19"/>
     </row>
     <row r="22" spans="1:6" ht="24" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C22" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D22" s="20" t="s">
-        <v>84</v>
-      </c>
-      <c r="E22" s="21"/>
-      <c r="F22" s="21"/>
+      <c r="D22" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="E22" s="19"/>
+      <c r="F22" s="19"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
@@ -1229,11 +1223,11 @@
       <c r="C23" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D23" s="22" t="s">
+      <c r="D23" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="E23" s="21"/>
-      <c r="F23" s="21"/>
+      <c r="E23" s="19"/>
+      <c r="F23" s="19"/>
     </row>
     <row r="24" spans="1:6" ht="24" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
@@ -1245,11 +1239,11 @@
       <c r="C24" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D24" s="20" t="s">
+      <c r="D24" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="21"/>
-      <c r="F24" s="21"/>
+      <c r="E24" s="19"/>
+      <c r="F24" s="19"/>
     </row>
     <row r="25" spans="1:6" ht="24" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
@@ -1261,19 +1255,14 @@
       <c r="C25" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D25" s="22" t="s">
+      <c r="D25" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="E25" s="21"/>
-      <c r="F25" s="21"/>
+      <c r="E25" s="19"/>
+      <c r="F25" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="D25:F25"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="D23:F23"/>
-    <mergeCell ref="D18:F18"/>
-    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="D24:F24"/>
     <mergeCell ref="D22:F22"/>
@@ -1282,6 +1271,11 @@
     <mergeCell ref="A18"/>
     <mergeCell ref="D19:F19"/>
     <mergeCell ref="D20:F20"/>
+    <mergeCell ref="D25:F25"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="D23:F23"/>
+    <mergeCell ref="D18:F18"/>
+    <mergeCell ref="A17:F17"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="8" orientation="portrait" r:id="rId1"/>

</xml_diff>